<commit_message>
Corrige eliminacao 20 na Rodada 10
</commit_message>
<xml_diff>
--- a/liga_eliminacao/datasets_liga_eliminacao/Pontuacoes_Por_Rodada_Liga_Eliminacao_20.xlsx
+++ b/liga_eliminacao/datasets_liga_eliminacao/Pontuacoes_Por_Rodada_Liga_Eliminacao_20.xlsx
@@ -76,7 +76,7 @@
     <t>Rodada 19</t>
   </si>
   <si>
-    <t>Parcial Rodada 11</t>
+    <t>Parcial Rodada 10</t>
   </si>
   <si>
     <t>time_id</t>
@@ -603,10 +603,10 @@
         <v>85.93994140625</v>
       </c>
       <c r="L2">
-        <v>43.590087890625</v>
-      </c>
-      <c r="M2">
-        <v>43.590087890625</v>
+        <v>85.93994140625</v>
+      </c>
+      <c r="V2">
+        <v>43.59</v>
       </c>
     </row>
     <row r="3" spans="1:22">
@@ -644,10 +644,10 @@
         <v>94.27978515625</v>
       </c>
       <c r="L3">
-        <v>70.77001953125</v>
-      </c>
-      <c r="M3">
-        <v>70.77001953125</v>
+        <v>94.27978515625</v>
+      </c>
+      <c r="V3">
+        <v>71.17</v>
       </c>
     </row>
     <row r="4" spans="1:22">
@@ -675,6 +675,9 @@
       <c r="H4">
         <v>47.389892578125</v>
       </c>
+      <c r="V4">
+        <v>39.87</v>
+      </c>
     </row>
     <row r="5" spans="1:22">
       <c r="A5" s="1">
@@ -689,6 +692,9 @@
       <c r="D5">
         <v>44.679931640625</v>
       </c>
+      <c r="V5">
+        <v>69.06999999999999</v>
+      </c>
     </row>
     <row r="6" spans="1:22">
       <c r="A6" s="1">
@@ -725,10 +731,10 @@
         <v>85.85009765625</v>
       </c>
       <c r="L6">
-        <v>58.090087890625</v>
-      </c>
-      <c r="M6">
-        <v>58.090087890625</v>
+        <v>85.85009765625</v>
+      </c>
+      <c r="V6">
+        <v>59.29</v>
       </c>
     </row>
     <row r="7" spans="1:22">
@@ -765,6 +771,9 @@
       <c r="K7">
         <v>39.699951171875</v>
       </c>
+      <c r="V7">
+        <v>32.15</v>
+      </c>
     </row>
     <row r="8" spans="1:22">
       <c r="A8" s="1">
@@ -801,7 +810,10 @@
         <v>49.760009765625</v>
       </c>
       <c r="L8">
-        <v>38.780029296875</v>
+        <v>49.760009765625</v>
+      </c>
+      <c r="V8">
+        <v>39.58</v>
       </c>
     </row>
     <row r="9" spans="1:22">
@@ -839,10 +851,10 @@
         <v>59.010009765625</v>
       </c>
       <c r="L9">
-        <v>60.169921875</v>
-      </c>
-      <c r="M9">
-        <v>60.169921875</v>
+        <v>59.010009765625</v>
+      </c>
+      <c r="V9">
+        <v>60.57</v>
       </c>
     </row>
     <row r="10" spans="1:22">
@@ -880,10 +892,10 @@
         <v>66.93994140625</v>
       </c>
       <c r="L10">
-        <v>58.949951171875</v>
-      </c>
-      <c r="M10">
-        <v>58.949951171875</v>
+        <v>66.93994140625</v>
+      </c>
+      <c r="V10">
+        <v>59.75</v>
       </c>
     </row>
     <row r="11" spans="1:22">
@@ -902,6 +914,9 @@
       <c r="E11">
         <v>42.14990234375</v>
       </c>
+      <c r="V11">
+        <v>19.4</v>
+      </c>
     </row>
     <row r="12" spans="1:22">
       <c r="A12" s="1">
@@ -938,10 +953,10 @@
         <v>70.10009765625</v>
       </c>
       <c r="L12">
-        <v>42.090087890625</v>
-      </c>
-      <c r="M12">
-        <v>42.090087890625</v>
+        <v>70.10009765625</v>
+      </c>
+      <c r="V12">
+        <v>42.89</v>
       </c>
     </row>
     <row r="13" spans="1:22">
@@ -954,6 +969,9 @@
       <c r="C13">
         <v>0</v>
       </c>
+      <c r="V13">
+        <v>67.78</v>
+      </c>
     </row>
     <row r="14" spans="1:22">
       <c r="A14" s="1">
@@ -990,10 +1008,10 @@
         <v>62.89990234375</v>
       </c>
       <c r="L14">
-        <v>43.25</v>
-      </c>
-      <c r="M14">
-        <v>43.25</v>
+        <v>62.89990234375</v>
+      </c>
+      <c r="V14">
+        <v>44.05</v>
       </c>
     </row>
     <row r="15" spans="1:22">
@@ -1018,6 +1036,9 @@
       <c r="G15">
         <v>41.169921875</v>
       </c>
+      <c r="V15">
+        <v>54.48</v>
+      </c>
     </row>
     <row r="16" spans="1:22">
       <c r="A16" s="1">
@@ -1047,8 +1068,11 @@
       <c r="I16">
         <v>48.469970703125</v>
       </c>
-    </row>
-    <row r="17" spans="1:13">
+      <c r="V16">
+        <v>55.58</v>
+      </c>
+    </row>
+    <row r="17" spans="1:22">
       <c r="A17" s="1">
         <v>19209079</v>
       </c>
@@ -1083,13 +1107,13 @@
         <v>87.14013671875</v>
       </c>
       <c r="L17">
-        <v>55.27001953125</v>
-      </c>
-      <c r="M17">
-        <v>55.27001953125</v>
-      </c>
-    </row>
-    <row r="18" spans="1:13">
+        <v>87.14013671875</v>
+      </c>
+      <c r="V17">
+        <v>56.47</v>
+      </c>
+    </row>
+    <row r="18" spans="1:22">
       <c r="A18" s="1">
         <v>19833277</v>
       </c>
@@ -1124,10 +1148,13 @@
         <v>73.68017578125</v>
       </c>
       <c r="L18">
-        <v>30.3699951171875</v>
-      </c>
-    </row>
-    <row r="19" spans="1:13">
+        <v>73.68017578125</v>
+      </c>
+      <c r="V18">
+        <v>31.57</v>
+      </c>
+    </row>
+    <row r="19" spans="1:22">
       <c r="A19" s="1">
         <v>20651178</v>
       </c>
@@ -1146,8 +1173,11 @@
       <c r="F19">
         <v>42.56005859375</v>
       </c>
-    </row>
-    <row r="20" spans="1:13">
+      <c r="V19">
+        <v>60.45</v>
+      </c>
+    </row>
+    <row r="20" spans="1:22">
       <c r="A20" s="1">
         <v>44810918</v>
       </c>
@@ -1182,13 +1212,13 @@
         <v>104.68017578125</v>
       </c>
       <c r="L20">
-        <v>66.89013671875</v>
-      </c>
-      <c r="M20">
-        <v>66.89013671875</v>
-      </c>
-    </row>
-    <row r="21" spans="1:13">
+        <v>104.68017578125</v>
+      </c>
+      <c r="V20">
+        <v>67.29000000000001</v>
+      </c>
+    </row>
+    <row r="21" spans="1:22">
       <c r="A21" s="1">
         <v>47775950</v>
       </c>
@@ -1218,6 +1248,9 @@
       </c>
       <c r="J21">
         <v>42.89990234375</v>
+      </c>
+      <c r="V21">
+        <v>66.56999999999999</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Corrige regra da eliminacao 20
</commit_message>
<xml_diff>
--- a/liga_eliminacao/datasets_liga_eliminacao/Pontuacoes_Por_Rodada_Liga_Eliminacao_20.xlsx
+++ b/liga_eliminacao/datasets_liga_eliminacao/Pontuacoes_Por_Rodada_Liga_Eliminacao_20.xlsx
@@ -76,7 +76,7 @@
     <t>Rodada 19</t>
   </si>
   <si>
-    <t>Parcial Rodada 10</t>
+    <t>Parcial Rodada 11</t>
   </si>
   <si>
     <t>time_id</t>
@@ -603,10 +603,10 @@
         <v>85.93994140625</v>
       </c>
       <c r="L2">
-        <v>85.93994140625</v>
-      </c>
-      <c r="V2">
-        <v>43.59</v>
+        <v>43.590087890625</v>
+      </c>
+      <c r="M2">
+        <v>43.590087890625</v>
       </c>
     </row>
     <row r="3" spans="1:22">
@@ -644,10 +644,10 @@
         <v>94.27978515625</v>
       </c>
       <c r="L3">
-        <v>94.27978515625</v>
-      </c>
-      <c r="V3">
-        <v>71.17</v>
+        <v>70.77001953125</v>
+      </c>
+      <c r="M3">
+        <v>70.77001953125</v>
       </c>
     </row>
     <row r="4" spans="1:22">
@@ -675,9 +675,6 @@
       <c r="H4">
         <v>47.389892578125</v>
       </c>
-      <c r="V4">
-        <v>39.87</v>
-      </c>
     </row>
     <row r="5" spans="1:22">
       <c r="A5" s="1">
@@ -692,9 +689,6 @@
       <c r="D5">
         <v>44.679931640625</v>
       </c>
-      <c r="V5">
-        <v>69.06999999999999</v>
-      </c>
     </row>
     <row r="6" spans="1:22">
       <c r="A6" s="1">
@@ -731,10 +725,10 @@
         <v>85.85009765625</v>
       </c>
       <c r="L6">
-        <v>85.85009765625</v>
-      </c>
-      <c r="V6">
-        <v>59.29</v>
+        <v>58.090087890625</v>
+      </c>
+      <c r="M6">
+        <v>58.090087890625</v>
       </c>
     </row>
     <row r="7" spans="1:22">
@@ -771,9 +765,6 @@
       <c r="K7">
         <v>39.699951171875</v>
       </c>
-      <c r="V7">
-        <v>32.15</v>
-      </c>
     </row>
     <row r="8" spans="1:22">
       <c r="A8" s="1">
@@ -810,10 +801,10 @@
         <v>49.760009765625</v>
       </c>
       <c r="L8">
-        <v>49.760009765625</v>
-      </c>
-      <c r="V8">
-        <v>39.58</v>
+        <v>38.780029296875</v>
+      </c>
+      <c r="M8">
+        <v>38.780029296875</v>
       </c>
     </row>
     <row r="9" spans="1:22">
@@ -851,10 +842,10 @@
         <v>59.010009765625</v>
       </c>
       <c r="L9">
-        <v>59.010009765625</v>
-      </c>
-      <c r="V9">
-        <v>60.57</v>
+        <v>60.169921875</v>
+      </c>
+      <c r="M9">
+        <v>60.169921875</v>
       </c>
     </row>
     <row r="10" spans="1:22">
@@ -892,10 +883,10 @@
         <v>66.93994140625</v>
       </c>
       <c r="L10">
-        <v>66.93994140625</v>
-      </c>
-      <c r="V10">
-        <v>59.75</v>
+        <v>58.949951171875</v>
+      </c>
+      <c r="M10">
+        <v>58.949951171875</v>
       </c>
     </row>
     <row r="11" spans="1:22">
@@ -914,9 +905,6 @@
       <c r="E11">
         <v>42.14990234375</v>
       </c>
-      <c r="V11">
-        <v>19.4</v>
-      </c>
     </row>
     <row r="12" spans="1:22">
       <c r="A12" s="1">
@@ -953,10 +941,10 @@
         <v>70.10009765625</v>
       </c>
       <c r="L12">
-        <v>70.10009765625</v>
-      </c>
-      <c r="V12">
-        <v>42.89</v>
+        <v>42.090087890625</v>
+      </c>
+      <c r="M12">
+        <v>42.090087890625</v>
       </c>
     </row>
     <row r="13" spans="1:22">
@@ -969,9 +957,6 @@
       <c r="C13">
         <v>0</v>
       </c>
-      <c r="V13">
-        <v>67.78</v>
-      </c>
     </row>
     <row r="14" spans="1:22">
       <c r="A14" s="1">
@@ -1008,10 +993,10 @@
         <v>62.89990234375</v>
       </c>
       <c r="L14">
-        <v>62.89990234375</v>
-      </c>
-      <c r="V14">
-        <v>44.05</v>
+        <v>43.25</v>
+      </c>
+      <c r="M14">
+        <v>43.25</v>
       </c>
     </row>
     <row r="15" spans="1:22">
@@ -1036,9 +1021,6 @@
       <c r="G15">
         <v>41.169921875</v>
       </c>
-      <c r="V15">
-        <v>54.48</v>
-      </c>
     </row>
     <row r="16" spans="1:22">
       <c r="A16" s="1">
@@ -1068,11 +1050,8 @@
       <c r="I16">
         <v>48.469970703125</v>
       </c>
-      <c r="V16">
-        <v>55.58</v>
-      </c>
-    </row>
-    <row r="17" spans="1:22">
+    </row>
+    <row r="17" spans="1:13">
       <c r="A17" s="1">
         <v>19209079</v>
       </c>
@@ -1107,13 +1086,13 @@
         <v>87.14013671875</v>
       </c>
       <c r="L17">
-        <v>87.14013671875</v>
-      </c>
-      <c r="V17">
-        <v>56.47</v>
-      </c>
-    </row>
-    <row r="18" spans="1:22">
+        <v>55.27001953125</v>
+      </c>
+      <c r="M17">
+        <v>55.27001953125</v>
+      </c>
+    </row>
+    <row r="18" spans="1:13">
       <c r="A18" s="1">
         <v>19833277</v>
       </c>
@@ -1148,13 +1127,10 @@
         <v>73.68017578125</v>
       </c>
       <c r="L18">
-        <v>73.68017578125</v>
-      </c>
-      <c r="V18">
-        <v>31.57</v>
-      </c>
-    </row>
-    <row r="19" spans="1:22">
+        <v>30.3699951171875</v>
+      </c>
+    </row>
+    <row r="19" spans="1:13">
       <c r="A19" s="1">
         <v>20651178</v>
       </c>
@@ -1173,11 +1149,8 @@
       <c r="F19">
         <v>42.56005859375</v>
       </c>
-      <c r="V19">
-        <v>60.45</v>
-      </c>
-    </row>
-    <row r="20" spans="1:22">
+    </row>
+    <row r="20" spans="1:13">
       <c r="A20" s="1">
         <v>44810918</v>
       </c>
@@ -1212,13 +1185,13 @@
         <v>104.68017578125</v>
       </c>
       <c r="L20">
-        <v>104.68017578125</v>
-      </c>
-      <c r="V20">
-        <v>67.29000000000001</v>
-      </c>
-    </row>
-    <row r="21" spans="1:22">
+        <v>66.89013671875</v>
+      </c>
+      <c r="M20">
+        <v>66.89013671875</v>
+      </c>
+    </row>
+    <row r="21" spans="1:13">
       <c r="A21" s="1">
         <v>47775950</v>
       </c>
@@ -1248,9 +1221,6 @@
       </c>
       <c r="J21">
         <v>42.89990234375</v>
-      </c>
-      <c r="V21">
-        <v>66.56999999999999</v>
       </c>
     </row>
   </sheetData>

</xml_diff>